<commit_message>
Update assessment details workbook
</commit_message>
<xml_diff>
--- a/AssessmentDetails.xlsx
+++ b/AssessmentDetails.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="156">
   <si>
     <t>Date</t>
   </si>
@@ -397,6 +397,218 @@
   </si>
   <si>
     <t>2026-06-29T05:31:10.559Z</t>
+  </si>
+  <si>
+    <t>18:50</t>
+  </si>
+  <si>
+    <t>test00007</t>
+  </si>
+  <si>
+    <t>1m 53s</t>
+  </si>
+  <si>
+    <t>82</t>
+  </si>
+  <si>
+    <t>Good performance! You showed strong knowledge with 89% accuracy, 91% confidence, and 64% communication skills.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Technical knowledge
+Clear thinking
+Problem-solving</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Technical depth
+Confidence
+Communication</t>
+  </si>
+  <si>
+    <t>Technical accuracy score: 89%. Continue strengthening topic depth and practical examples.</t>
+  </si>
+  <si>
+    <t>Communication score: 64%. Keep answers structured, concise, and example driven.</t>
+  </si>
+  <si>
+    <t>Confidence score: 91%. Continue improving clarity, conviction, and professional interview presence.</t>
+  </si>
+  <si>
+    <t>Continue practicing and building your technical expertise.</t>
+  </si>
+  <si>
+    <t>/Users/nandhakumar_r/Documents/CodeGen/InterviewBot/AIInterviewAgestWithTraining/AIInterviewAgent29June26-6pm/reports/Report_test00007_2026-06-29T13-23-14-088Z.pdf</t>
+  </si>
+  <si>
+    <t>2026-06-29T13:22:22.210Z</t>
+  </si>
+  <si>
+    <t>19:04</t>
+  </si>
+  <si>
+    <t>test1234</t>
+  </si>
+  <si>
+    <t>14s</t>
+  </si>
+  <si>
+    <t>79</t>
+  </si>
+  <si>
+    <t>Competent</t>
+  </si>
+  <si>
+    <t>Good performance! You showed strong knowledge with 94% accuracy, 60% confidence, and 84% communication skills.</t>
+  </si>
+  <si>
+    <t>Technical accuracy score: 94%. Continue strengthening topic depth and practical examples.</t>
+  </si>
+  <si>
+    <t>Communication score: 84%. Keep answers structured, concise, and example driven.</t>
+  </si>
+  <si>
+    <t>Confidence score: 60%. Continue improving clarity, conviction, and professional interview presence.</t>
+  </si>
+  <si>
+    <t>Completed - Passed</t>
+  </si>
+  <si>
+    <t>/Users/nandhakumar_r/Documents/CodeGen/InterviewBot/AIInterviewAgestWithTraining/AIInterviewAgent29June26-6pm/reports/Report_test1234_2026-06-29T13-35-21-830Z.pdf</t>
+  </si>
+  <si>
+    <t>2026-06-29T13:35:15.503Z</t>
+  </si>
+  <si>
+    <t>19:19</t>
+  </si>
+  <si>
+    <t>11s</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>AI evaluation was unavailable or incomplete (OpenAI API error). Objective questions were scored using their answer keys, and descriptive answers are included for manual review. The candidate completed 2 questions. Final marks are based on validated technical correctness, while confidence and communication are shown as supporting signals.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Completed the interview flow
+Provided responses for the captured questions
+Demonstrated areas that can now be reviewed question by question</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Increase answer depth with implementation details
+Use examples, tradeoffs, and edge cases
+Keep responses structured around the exact question asked</t>
+  </si>
+  <si>
+    <t>AI evaluation was unavailable or incomplete (OpenAI API error). Objective questions were scored using their answer keys, and descriptive answers are included for manual review. Technical correctness is calculated from the detailed question evaluations below. Review each answer for exact concepts, missed points, and expected rubric alignment.</t>
+  </si>
+  <si>
+    <t>Communication was estimated from answer completeness and clarity. Strong answers should define the concept, explain why it matters, and finish with a practical example.</t>
+  </si>
+  <si>
+    <t>Professional readiness should be assessed from consistency, focus, and interview discipline. Tab switches: 0. Time outside: 0 seconds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Question 1: Explain how you would approach Banking react-native Project using react-native.
+Candidate Answer: ok
+Assessment: Needs Review (Needs review)
+Expected Answer / Rubric: Customer profile: DFB Customer - Banking react-native Project
+Technology: react-native
+Role level: senior
+Expected points: architecture, project context, tradeoffs
+Feedback: The answer has been captured, but automatic AI validation was unavailable or incomplete for this descriptive question. Expected answer or rubric: Customer profile: DFB Customer - Banking react-native Project Technology: react-native Role level: senior Expected points: architecture, project context, tradeoffs. A reviewer should compare the response against the rubric and check for correctness, depth, examples, and missing edge cases.
+Missing Concepts: Add more precise technical detail
+Include a practical example or edge case
+Improvement Suggestion: Rewrite the answer with the main concept first, then add implementation details, tradeoffs, and a concise example.
+Question 2: What are the top security considerations for a Banking application?
+Candidate Answer: no
+Assessment: Needs Review (Needs review)
+Expected Answer / Rubric: Customer profile: DFB Customer - Banking react-native Project
+Technology: react-native
+Role level: senior
+Expected points: security, compliance, data protection
+Feedback: The answer has been captured, but automatic AI validation was unavailable or incomplete for this descriptive question. Expected answer or rubric: Customer profile: DFB Customer - Banking react-native Project Technology: react-native Role level: senior Expected points: security, compliance, data protection. A reviewer should compare the response against the rubric and check for correctness, depth, examples, and missing edge cases.
+Missing Concepts: Add more precise technical detail
+Include a practical example or edge case
+Improvement Suggestion: Rewrite the answer with the main concept first, then add implementation details, tradeoffs, and a concise example.</t>
+  </si>
+  <si>
+    <t>Review every incorrect or partially correct answer, rewrite it with the expected concept and a practical example, then repeat a timed mock interview.</t>
+  </si>
+  <si>
+    <t>/Users/nandhakumar_r/Documents/CodeGen/InterviewBot/AIInterviewAgestWithTraining/AIInterviewAgent29June26-6pm/reports/Report_test1234_2026-06-29T13-50-32-096Z.pdf</t>
+  </si>
+  <si>
+    <t>2026-06-29T13:50:14.869Z</t>
+  </si>
+  <si>
+    <t>30/06/2026</t>
+  </si>
+  <si>
+    <t>08:41</t>
+  </si>
+  <si>
+    <t>test090</t>
+  </si>
+  <si>
+    <t>21s</t>
+  </si>
+  <si>
+    <t>AI evaluation was unavailable or incomplete (Error evaluating assessment report). Objective questions were scored using their answer keys, and descriptive answers are included for manual review. The candidate completed 3 questions. Final marks are based on validated technical correctness, while confidence and communication are shown as supporting signals.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Completed the interview flow
+Provided responses for the captured questions
+Demonstrated areas that can now be reviewed question by question</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Increase answer depth with implementation details
+Use examples, tradeoffs, and edge cases
+Keep responses structured around the exact question asked</t>
+  </si>
+  <si>
+    <t>AI evaluation was unavailable or incomplete (Error evaluating assessment report). Objective questions were scored using their answer keys, and descriptive answers are included for manual review. Technical correctness is calculated from the detailed question evaluations below. Review each answer for exact concepts, missed points, and expected rubric alignment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Question 1: Explain how you would approach Banking react-native Project using react-native.
+Candidate Answer: ds
+Assessment: Needs Review (Needs review)
+Expected Answer / Rubric: Customer profile: DFB Customer - Banking react-native Project
+Technology: react-native
+Role level: senior
+Expected points: architecture, project context, tradeoffs
+Feedback: The answer has been captured, but automatic AI validation was unavailable or incomplete for this descriptive question. Expected answer or rubric: Customer profile: DFB Customer - Banking react-native Project Technology: react-native Role level: senior Expected points: architecture, project context, tradeoffs. A reviewer should compare the response against the rubric and check for correctness, depth, examples, and missing edge cases.
+Missing Concepts: Add more precise technical detail
+Include a practical example or edge case
+Improvement Suggestion: Rewrite the answer with the main concept first, then add implementation details, tradeoffs, and a concise example.
+Question 2: Tell us about a time you used feedback or metrics to improve a technical delivery outcome.
+Candidate Answer: ds
+Assessment: Needs Review (Needs review)
+Expected Answer / Rubric: Customer profile: DFB Customer - Banking react-native Project
+Technology: react-native
+Role level: senior
+Expected points: metrics, ownership, continuous improvement
+Feedback: The answer has been captured, but automatic AI validation was unavailable or incomplete for this descriptive question. Expected answer or rubric: Customer profile: DFB Customer - Banking react-native Project Technology: react-native Role level: senior Expected points: metrics, ownership, continuous improvement. A reviewer should compare the response against the rubric and check for correctness, depth, examples, and missing edge cases.
+Missing Concepts: Add more precise technical detail
+Include a practical example or edge case
+Improvement Suggestion: Rewrite the answer with the main concept first, then add implementation details, tradeoffs, and a concise example.
+Question 3: How would you validate that the interview focus areas for DFB Customer are still aligned with current project needs?
+Candidate Answer: ds
+Assessment: Needs Review (Needs review)
+Expected Answer / Rubric: Customer profile: DFB Customer - Banking react-native Project
+Technology: react-native
+Role level: senior
+Expected points: customer requirements, feedback loop, quality checks
+Feedback: The answer has been captured, but automatic AI validation was unavailable or incomplete for this descriptive question. Expected answer or rubric: Customer profile: DFB Customer - Banking react-native Project Technology: react-native Role level: senior Expected points: customer requirements, feedback loop, quality checks. A reviewer should compare the response against the rubric and check for correctness, depth, examples, and missing edge cases.
+Missing Concepts: Add more precise technical detail
+Include a practical example or edge case
+Improvement Suggestion: Rewrite the answer with the main concept first, then add implementation details, tradeoffs, and a concise example.</t>
+  </si>
+  <si>
+    <t>/Users/nandhakumar_r/Documents/CodeGen/InterviewBot/AIInterviewAgestWithTraining/AIInterviewAgent29June26-6pm/reports/Report_test090_2026-06-30T03-12-37-670Z.pdf</t>
+  </si>
+  <si>
+    <t>2026-06-30T03:12:21.941Z</t>
   </si>
 </sst>
 </file>
@@ -794,7 +1006,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:W9"/>
+  <dimension ref="A1:W13"/>
   <sheetFormatPr defaultRowHeight="16" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1456,11 +1668,299 @@
         <v>106</v>
       </c>
     </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M10" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="N10" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="O10" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="P10" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q10" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="R10" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="S10" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="T10" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="U10" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="V10" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="W10" s="4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="M11" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="N11" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="O11" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="P11" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="Q11" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="R11" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="S11" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="T11" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="U11" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="V11" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="W11" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="M12" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="N12" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="O12" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="P12" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q12" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="R12" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="S12" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="T12" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="U12" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="V12" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="W12" s="4" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="M13" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="N13" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="O13" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="P13" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q13" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="R13" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="S13" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="T13" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="U13" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="V13" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="W13" s="4" t="s">
+        <v>155</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="V7" r:id="rId1"/>
     <hyperlink ref="V8" r:id="rId2"/>
     <hyperlink ref="V9" r:id="rId3"/>
+    <hyperlink ref="V10" r:id="rId4"/>
+    <hyperlink ref="V11" r:id="rId5"/>
+    <hyperlink ref="V12" r:id="rId6"/>
+    <hyperlink ref="V13" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>